<commit_message>
BCDecoder16Combinations & Fix TrueTable Added
</commit_message>
<xml_diff>
--- a/Team14_Lab4/TrueTable_BcdDecoder.xlsx
+++ b/Team14_Lab4/TrueTable_BcdDecoder.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Quartus_Labs\Team14_Lab4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Quartus_Labs\Fundamentals_Of_Digital_Design_FPGA\Team14_Lab4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E960681-C0BD-49B4-9859-B96A1AA551DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00573712-EF8B-43A8-B655-23CBB2F45AD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{6B52F0DE-526B-4DF2-A948-F7CE809520DF}"/>
   </bookViews>
@@ -141,19 +141,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -186,6 +180,24 @@
       <color theme="1"/>
       <name val="Amasis MT Pro Medium"/>
       <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="10"/>
+      <name val="Amasis MT Pro Medium"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -356,18 +368,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -376,34 +388,43 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -757,41 +778,41 @@
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="11" t="s">
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="12"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="14"/>
     </row>
     <row r="2" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="13"/>
-      <c r="B2" s="14"/>
+      <c r="A2" s="10"/>
+      <c r="B2" s="12"/>
       <c r="C2" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="16" t="s">
+      <c r="I2" s="8" t="s">
         <v>8</v>
       </c>
     </row>
@@ -802,13 +823,13 @@
       <c r="B3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="16">
         <v>1</v>
       </c>
       <c r="D3" s="5">
         <v>1</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="16">
         <v>1</v>
       </c>
       <c r="F3" s="5">
@@ -831,13 +852,13 @@
       <c r="B4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="17">
         <v>0</v>
       </c>
       <c r="D4" s="6">
         <v>1</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="17">
         <v>1</v>
       </c>
       <c r="F4" s="6">
@@ -860,13 +881,13 @@
       <c r="B5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="17">
         <v>1</v>
       </c>
       <c r="D5" s="6">
         <v>1</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="17">
         <v>0</v>
       </c>
       <c r="F5" s="6">
@@ -889,13 +910,13 @@
       <c r="B6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="17">
         <v>1</v>
       </c>
       <c r="D6" s="6">
         <v>1</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="18" t="s">
         <v>32</v>
       </c>
       <c r="F6" s="6">
@@ -918,13 +939,13 @@
       <c r="B7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="17">
         <v>0</v>
       </c>
       <c r="D7" s="6">
         <v>1</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="17">
         <v>1</v>
       </c>
       <c r="F7" s="6">
@@ -947,13 +968,13 @@
       <c r="B8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="17">
         <v>1</v>
       </c>
       <c r="D8" s="6">
         <v>0</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="19">
         <v>1</v>
       </c>
       <c r="F8" s="6">
@@ -976,13 +997,13 @@
       <c r="B9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="17">
         <v>1</v>
       </c>
       <c r="D9" s="6">
         <v>0</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="17">
         <v>1</v>
       </c>
       <c r="F9" s="6">
@@ -1005,13 +1026,13 @@
       <c r="B10" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="17">
         <v>1</v>
       </c>
       <c r="D10" s="6">
         <v>1</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="17">
         <v>1</v>
       </c>
       <c r="F10" s="6">
@@ -1034,13 +1055,13 @@
       <c r="B11" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="17">
         <v>1</v>
       </c>
       <c r="D11" s="6">
         <v>1</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="17">
         <v>1</v>
       </c>
       <c r="F11" s="6">
@@ -1063,13 +1084,13 @@
       <c r="B12" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="17">
         <v>1</v>
       </c>
       <c r="D12" s="6">
         <v>1</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="17">
         <v>1</v>
       </c>
       <c r="F12" s="6">
@@ -1092,13 +1113,13 @@
       <c r="B13" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="17">
         <v>1</v>
       </c>
       <c r="D13" s="6">
         <v>1</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="17">
         <v>1</v>
       </c>
       <c r="F13" s="6">
@@ -1121,13 +1142,13 @@
       <c r="B14" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="17">
         <v>0</v>
       </c>
       <c r="D14" s="6">
         <v>0</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="17">
         <v>1</v>
       </c>
       <c r="F14" s="6">
@@ -1150,14 +1171,14 @@
       <c r="B15" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="6">
-        <v>0</v>
+      <c r="C15" s="17">
+        <v>1</v>
       </c>
       <c r="D15" s="6">
         <v>0</v>
       </c>
-      <c r="E15" s="6">
-        <v>1</v>
+      <c r="E15" s="17">
+        <v>0</v>
       </c>
       <c r="F15" s="6">
         <v>1</v>
@@ -1179,13 +1200,13 @@
       <c r="B16" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="6">
+      <c r="C16" s="17">
         <v>0</v>
       </c>
       <c r="D16" s="6">
         <v>1</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="17">
         <v>1</v>
       </c>
       <c r="F16" s="6">
@@ -1208,13 +1229,13 @@
       <c r="B17" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="17">
         <v>1</v>
       </c>
       <c r="D17" s="6">
         <v>0</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="17">
         <v>0</v>
       </c>
       <c r="F17" s="6">
@@ -1237,13 +1258,13 @@
       <c r="B18" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="17">
         <v>1</v>
       </c>
       <c r="D18" s="6">
         <v>0</v>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="17">
         <v>0</v>
       </c>
       <c r="F18" s="6">

</xml_diff>